<commit_message>
data: publish 2026-09-16 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-16-182路.xlsx
+++ b/data/export/2026-09-16-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC23"/>
+  <dimension ref="A1:AC39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,22 +708,22 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>88.0</t>
+          <t>81.3</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -827,22 +827,22 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>85.0</t>
+          <t>77.7</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -946,22 +946,22 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>84.0</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1065,22 +1065,22 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>80.5</t>
+          <t>80.7</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>1/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1184,22 +1184,22 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
-          <t>88.0</t>
+          <t>83.3</t>
         </is>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>12/14</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA7" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>91.0</t>
+          <t>79.7</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -1356,12 +1356,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:27</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>91分钟</t>
+          <t>92分钟</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1422,22 +1422,22 @@
       </c>
       <c r="Z8" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA8" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
-          <t>91.0</t>
+          <t>83.0</t>
         </is>
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -1470,27 +1470,31 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>08:29</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>91分钟</t>
+          <t>89分钟</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS末次终点ETA推算：08:11采样，终点ETA 19分钟</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
           <t>06:21</t>
@@ -1498,7 +1502,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1522,12 +1526,12 @@
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>末次终点ETA兜底</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
@@ -1542,17 +1546,17 @@
       </c>
       <c r="AA9" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
-          <t>91.0</t>
+          <t>80.5</t>
         </is>
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1585,27 +1589,31 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:42</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>90分钟</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
           <t>06:41</t>
@@ -1613,7 +1621,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1637,33 +1645,37 @@
       </c>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA10" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB10" s="2" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr">
+        <is>
+          <t>80.7</t>
+        </is>
+      </c>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>—/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -1696,24 +1708,24 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:53</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>96分钟</t>
+          <t>98分钟</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>08:01采样：该车到重点站华夏三路新德西路 ETA 35分钟；叠加该车自身同类时段从该站到终点历史中位数15分钟，约±5分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1728,7 +1740,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1752,12 +1764,12 @@
       </c>
       <c r="W11" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
@@ -1767,22 +1779,22 @@
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>96.0</t>
+          <t>80.0</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -1815,29 +1827,29 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>101分钟</t>
+          <t>99分钟</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>08:11采样：该车到重点站唐陆公路唐龙路 ETA 0分钟；叠加该车自身同类时段从该站到终点历史中位数53分钟，约±7分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1847,7 +1859,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1871,12 +1883,12 @@
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -1886,22 +1898,22 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>101.0</t>
+          <t>86.0</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>13/14</t>
         </is>
       </c>
     </row>
@@ -1934,29 +1946,29 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>09:12</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>98分钟</t>
+          <t>90分钟</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>08:11采样：该车到重点站东陆路新金桥路 ETA 1分钟；叠加该车自身同类时段从该站到终点历史中位数60分钟，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1966,7 +1978,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1990,12 +2002,12 @@
       </c>
       <c r="W13" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr">
@@ -2005,22 +2017,22 @@
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>88.0</t>
+          <t>81.3</t>
         </is>
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -2053,27 +2065,31 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:22</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>106分钟</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
           <t>07:11</t>
@@ -2081,7 +2097,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2105,33 +2121,37 @@
       </c>
       <c r="W14" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y14" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA14" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB14" s="2" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>82.3</t>
+        </is>
+      </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>—/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -2164,27 +2184,31 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>95分钟</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
           <t>07:21</t>
@@ -2192,7 +2216,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2216,33 +2240,37 @@
       </c>
       <c r="W15" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA15" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>95.0</t>
+        </is>
+      </c>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>—/14</t>
+          <t>14/14</t>
         </is>
       </c>
     </row>
@@ -2280,26 +2308,22 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>90分钟</t>
+          <t>92分钟</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数90分钟估算，约±5分钟</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+          <t>SHMAAS末次终点ETA推算：09:11采样，终点ETA 15分钟</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -2307,7 +2331,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2336,7 +2360,7 @@
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>末次终点ETA兜底</t>
         </is>
       </c>
       <c r="Y16" s="2" t="inlineStr">
@@ -2346,22 +2370,22 @@
       </c>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA16" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
-          <t>84.0</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -2394,29 +2418,29 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>94分钟</t>
+          <t>83分钟</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数94分钟估算，约±6分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -2426,7 +2450,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2450,12 +2474,12 @@
       </c>
       <c r="W17" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y17" s="2" t="inlineStr">
@@ -2465,22 +2489,22 @@
       </c>
       <c r="Z17" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA17" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>85.0</t>
+          <t>77.7</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -2513,29 +2537,29 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>09:29</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>74分钟</t>
+          <t>85分钟</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数74分钟估算，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -2545,7 +2569,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2569,12 +2593,12 @@
       </c>
       <c r="W18" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y18" s="2" t="inlineStr">
@@ -2584,22 +2608,22 @@
       </c>
       <c r="Z18" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA18" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
-          <t>80.5</t>
+          <t>80.7</t>
         </is>
       </c>
       <c r="AC18" s="2" t="inlineStr">
         <is>
-          <t>1/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -2632,12 +2656,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -2649,12 +2673,12 @@
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数86分钟估算，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -2664,7 +2688,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2688,12 +2712,12 @@
       </c>
       <c r="W19" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X19" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y19" s="2" t="inlineStr">
@@ -2703,22 +2727,22 @@
       </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA19" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
-          <t>88.0</t>
+          <t>83.3</t>
         </is>
       </c>
       <c r="AC19" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>12/14</t>
         </is>
       </c>
     </row>
@@ -2751,27 +2775,31 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>80分钟</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
           <t>07:51</t>
@@ -2779,7 +2807,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2803,33 +2831,37 @@
       </c>
       <c r="W20" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y20" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB20" s="2" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB20" s="2" t="inlineStr">
+        <is>
+          <t>73.5</t>
+        </is>
+      </c>
       <c r="AC20" s="2" t="inlineStr">
         <is>
-          <t>—/14</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -2867,26 +2899,22 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>96分钟</t>
+          <t>80分钟</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数96分钟估算，约±7分钟</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
+          <t>SHMAAS末次终点ETA推算：09:31采样，终点ETA 23分钟</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr">
         <is>
           <t>06:11</t>
@@ -2894,7 +2922,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2918,12 +2946,12 @@
       </c>
       <c r="W21" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>末次终点ETA兜底</t>
         </is>
       </c>
       <c r="Y21" s="2" t="inlineStr">
@@ -2933,22 +2961,22 @@
       </c>
       <c r="Z21" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA21" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
-          <t>91.0</t>
+          <t>79.7</t>
         </is>
       </c>
       <c r="AC21" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -2981,27 +3009,31 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>74分钟</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -3009,7 +3041,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3033,37 +3065,37 @@
       </c>
       <c r="W22" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y22" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z22" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA22" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA22" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
-          <t>91.0</t>
+          <t>83.0</t>
         </is>
       </c>
       <c r="AC22" s="2" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -3096,27 +3128,31 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>10:07</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
           <t>06:21</t>
@@ -3124,7 +3160,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -3148,37 +3184,1925 @@
       </c>
       <c r="W23" s="2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z23" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB23" s="2" t="inlineStr">
+        <is>
+          <t>80.5</t>
+        </is>
+      </c>
+      <c r="AC23" s="2" t="inlineStr">
+        <is>
+          <t>5/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>78分钟</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="inlineStr"/>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y24" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB24" s="2" t="inlineStr">
+        <is>
+          <t>80.7</t>
+        </is>
+      </c>
+      <c r="AC24" s="2" t="inlineStr">
+        <is>
+          <t>6/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>72分钟</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr"/>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y25" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA25" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB25" s="2" t="inlineStr">
+        <is>
+          <t>80.0</t>
+        </is>
+      </c>
+      <c r="AC25" s="2" t="inlineStr">
+        <is>
+          <t>4/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>09:22</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>73分钟</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>09:22</t>
+        </is>
+      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z26" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA26" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB26" s="2" t="inlineStr">
+        <is>
+          <t>86.0</t>
+        </is>
+      </c>
+      <c r="AC26" s="2" t="inlineStr">
+        <is>
+          <t>13/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>10:46</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>76分钟</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="inlineStr"/>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB27" s="2" t="inlineStr">
+        <is>
+          <t>81.3</t>
+        </is>
+      </c>
+      <c r="AC27" s="2" t="inlineStr">
+        <is>
+          <t>9/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>10:46</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>71分钟</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS末次终点ETA推算：10:32采样，终点ETA 14分钟</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr"/>
+      <c r="T28" s="2" t="inlineStr"/>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>末次终点ETA兜底</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA28" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB28" s="2" t="inlineStr">
+        <is>
+          <t>82.3</t>
+        </is>
+      </c>
+      <c r="AC28" s="2" t="inlineStr">
+        <is>
+          <t>10/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>沪A02126A</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X23" s="2" t="inlineStr">
+      <c r="X29" s="2" t="inlineStr">
         <is>
           <t>证据不足</t>
         </is>
       </c>
-      <c r="Y23" s="2" t="inlineStr">
+      <c r="Y29" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="Z23" s="2" t="inlineStr">
+      <c r="Z29" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA23" s="2" t="inlineStr">
+      <c r="AA29" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AB23" s="2" t="inlineStr">
-        <is>
-          <t>91.0</t>
-        </is>
-      </c>
-      <c r="AC23" s="2" t="inlineStr">
+      <c r="AB29" s="2" t="inlineStr">
+        <is>
+          <t>95.0</t>
+        </is>
+      </c>
+      <c r="AC29" s="2" t="inlineStr">
+        <is>
+          <t>14/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>11:03</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>73分钟</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS末次终点ETA推算：10:32采样，终点ETA 31分钟</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr"/>
+      <c r="T30" s="2" t="inlineStr"/>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>末次终点ETA兜底</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB30" s="2" t="inlineStr">
+        <is>
+          <t>81.0</t>
+        </is>
+      </c>
+      <c r="AC30" s="2" t="inlineStr">
+        <is>
+          <t>8/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>74分钟</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>10:32采样：该车到重点站唐陆公路锦绣东路 ETA 9分钟；叠加该车自身同类时段从该站到终点历史中位数38分钟，约±6分钟</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr"/>
+      <c r="S31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="inlineStr"/>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X31" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y31" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB31" s="2" t="inlineStr">
+        <is>
+          <t>77.7</t>
+        </is>
+      </c>
+      <c r="AC31" s="2" t="inlineStr">
+        <is>
+          <t>2/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>70分钟</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>10:21采样：该车到重点站德川路华夏东路 ETA 16分钟；叠加该车自身同类时段从该站到终点历史中位数48分钟，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr"/>
+      <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="inlineStr"/>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y32" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z32" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA32" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB32" s="2" t="inlineStr">
+        <is>
+          <t>80.7</t>
+        </is>
+      </c>
+      <c r="AC32" s="2" t="inlineStr">
         <is>
           <t>6/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>74分钟</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>10:21采样：该车到重点站博兴路东陆路 ETA 16分钟；叠加该车自身同类时段从该站到终点历史中位数56分钟，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr"/>
+      <c r="S33" s="2" t="inlineStr"/>
+      <c r="T33" s="2" t="inlineStr"/>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="V33" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W33" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X33" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y33" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z33" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA33" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB33" s="2" t="inlineStr">
+        <is>
+          <t>83.3</t>
+        </is>
+      </c>
+      <c r="AC33" s="2" t="inlineStr">
+        <is>
+          <t>12/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>沪A08953A</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>67分钟</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数67分钟估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="inlineStr"/>
+      <c r="T34" s="2" t="inlineStr"/>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="V34" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X34" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y34" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z34" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA34" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB34" s="2" t="inlineStr">
+        <is>
+          <t>73.5</t>
+        </is>
+      </c>
+      <c r="AC34" s="2" t="inlineStr">
+        <is>
+          <t>1/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr"/>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>73分钟</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数73分钟估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="inlineStr"/>
+      <c r="R35" s="2" t="inlineStr"/>
+      <c r="S35" s="2" t="inlineStr"/>
+      <c r="T35" s="2" t="inlineStr"/>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="V35" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W35" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X35" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y35" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z35" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA35" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB35" s="2" t="inlineStr">
+        <is>
+          <t>79.7</t>
+        </is>
+      </c>
+      <c r="AC35" s="2" t="inlineStr">
+        <is>
+          <t>3/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr"/>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>沪A31963D</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr"/>
+      <c r="R36" s="2" t="inlineStr"/>
+      <c r="S36" s="2" t="inlineStr"/>
+      <c r="T36" s="2" t="inlineStr"/>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="V36" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W36" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X36" s="2" t="inlineStr">
+        <is>
+          <t>证据不足</t>
+        </is>
+      </c>
+      <c r="Y36" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z36" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA36" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB36" s="2" t="inlineStr">
+        <is>
+          <t>83.0</t>
+        </is>
+      </c>
+      <c r="AC36" s="2" t="inlineStr">
+        <is>
+          <t>11/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>12:19</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>74分钟</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数74分钟估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q37" s="2" t="inlineStr"/>
+      <c r="R37" s="2" t="inlineStr"/>
+      <c r="S37" s="2" t="inlineStr"/>
+      <c r="T37" s="2" t="inlineStr"/>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="V37" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W37" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X37" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y37" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA37" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB37" s="2" t="inlineStr">
+        <is>
+          <t>80.7</t>
+        </is>
+      </c>
+      <c r="AC37" s="2" t="inlineStr">
+        <is>
+          <t>6/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr"/>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>70分钟</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数70分钟估算，约±12分钟</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="inlineStr"/>
+      <c r="R38" s="2" t="inlineStr"/>
+      <c r="S38" s="2" t="inlineStr"/>
+      <c r="T38" s="2" t="inlineStr"/>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="V38" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W38" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X38" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y38" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z38" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA38" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB38" s="2" t="inlineStr">
+        <is>
+          <t>80.0</t>
+        </is>
+      </c>
+      <c r="AC38" s="2" t="inlineStr">
+        <is>
+          <t>4/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr"/>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>70分钟</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数70分钟估算，约±7分钟</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="R39" s="2" t="inlineStr"/>
+      <c r="S39" s="2" t="inlineStr"/>
+      <c r="T39" s="2" t="inlineStr"/>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="V39" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W39" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y39" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB39" s="2" t="inlineStr">
+        <is>
+          <t>82.3</t>
+        </is>
+      </c>
+      <c r="AC39" s="2" t="inlineStr">
+        <is>
+          <t>10/14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-09-16 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-16-182路.xlsx
+++ b/data/export/2026-09-16-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC87"/>
+  <dimension ref="A1:AC98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,22 +708,22 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>80.4</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -837,12 +837,12 @@
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>79.9</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>9/15</t>
+          <t>8/15</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -946,22 +946,22 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>77.9</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>4/15</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1070,17 +1070,17 @@
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>78.6</t>
+          <t>81.8</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>6/15</t>
+          <t>13/15</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1184,22 +1184,22 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>82.7</t>
         </is>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>14/15</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA7" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>5/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>8/15</t>
+          <t>9/15</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>13/15</t>
+          <t>12/15</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1660,22 +1660,22 @@
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA10" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>7/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1740,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1779,22 +1779,22 @@
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>4/15</t>
+          <t>1/15</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1903,12 +1903,12 @@
       </c>
       <c r="AA12" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>83.8</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2017,22 +2017,22 @@
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>80.4</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2136,22 +2136,22 @@
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA14" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
-          <t>80.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>14/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2260,17 +2260,17 @@
       </c>
       <c r="AA15" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>77.2</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>2/15</t>
+          <t>3/15</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2370,22 +2370,22 @@
       </c>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA16" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>77.9</t>
         </is>
       </c>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>4/15</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2499,12 +2499,12 @@
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>79.9</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>9/15</t>
+          <t>8/15</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2569,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2613,17 +2613,17 @@
       </c>
       <c r="AA18" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
-          <t>78.6</t>
+          <t>81.8</t>
         </is>
       </c>
       <c r="AC18" s="2" t="inlineStr">
         <is>
-          <t>6/15</t>
+          <t>13/15</t>
         </is>
       </c>
     </row>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2727,22 +2727,22 @@
       </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA19" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>82.7</t>
         </is>
       </c>
       <c r="AC19" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>14/15</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2846,22 +2846,22 @@
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="AC20" s="2" t="inlineStr">
         <is>
-          <t>1/15</t>
+          <t>2/15</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2961,22 +2961,22 @@
       </c>
       <c r="Z21" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA21" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC21" s="2" t="inlineStr">
         <is>
-          <t>5/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="AC22" s="2" t="inlineStr">
         <is>
-          <t>8/15</t>
+          <t>9/15</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="AC23" s="2" t="inlineStr">
         <is>
-          <t>13/15</t>
+          <t>12/15</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3318,22 +3318,22 @@
       </c>
       <c r="Z24" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA24" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC24" s="2" t="inlineStr">
         <is>
-          <t>7/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3437,22 +3437,22 @@
       </c>
       <c r="Z25" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA25" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="AC25" s="2" t="inlineStr">
         <is>
-          <t>4/15</t>
+          <t>1/15</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3561,12 +3561,12 @@
       </c>
       <c r="AA26" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
-          <t>83.8</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="AC26" s="2" t="inlineStr">
@@ -3636,7 +3636,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3675,22 +3675,22 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA27" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
-          <t>80.4</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC27" s="2" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3790,22 +3790,22 @@
       </c>
       <c r="Z28" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA28" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
-          <t>80.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC28" s="2" t="inlineStr">
         <is>
-          <t>14/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3914,17 +3914,17 @@
       </c>
       <c r="AA29" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>77.2</t>
         </is>
       </c>
       <c r="AC29" s="2" t="inlineStr">
         <is>
-          <t>2/15</t>
+          <t>3/15</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -4028,22 +4028,22 @@
       </c>
       <c r="Z30" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA30" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>77.9</t>
         </is>
       </c>
       <c r="AC30" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>4/15</t>
         </is>
       </c>
     </row>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -4157,12 +4157,12 @@
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
-          <t>79.9</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="AC31" s="2" t="inlineStr">
         <is>
-          <t>9/15</t>
+          <t>8/15</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -4271,17 +4271,17 @@
       </c>
       <c r="AA32" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
-          <t>78.6</t>
+          <t>81.8</t>
         </is>
       </c>
       <c r="AC32" s="2" t="inlineStr">
         <is>
-          <t>6/15</t>
+          <t>13/15</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4346,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -4385,22 +4385,22 @@
       </c>
       <c r="Z33" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA33" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>82.7</t>
         </is>
       </c>
       <c r="AC33" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>14/15</t>
         </is>
       </c>
     </row>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -4504,22 +4504,22 @@
       </c>
       <c r="Z34" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA34" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="AC34" s="2" t="inlineStr">
         <is>
-          <t>1/15</t>
+          <t>2/15</t>
         </is>
       </c>
     </row>
@@ -4584,7 +4584,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -4623,22 +4623,22 @@
       </c>
       <c r="Z35" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA35" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC35" s="2" t="inlineStr">
         <is>
-          <t>5/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4757,7 @@
       </c>
       <c r="AC36" s="2" t="inlineStr">
         <is>
-          <t>8/15</t>
+          <t>9/15</t>
         </is>
       </c>
     </row>
@@ -4822,7 +4822,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -4861,22 +4861,22 @@
       </c>
       <c r="Z37" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA37" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC37" s="2" t="inlineStr">
         <is>
-          <t>7/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -4980,22 +4980,22 @@
       </c>
       <c r="Z38" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA38" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="AC38" s="2" t="inlineStr">
         <is>
-          <t>4/15</t>
+          <t>1/15</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -5099,22 +5099,22 @@
       </c>
       <c r="Z39" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA39" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
-          <t>80.4</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC39" s="2" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -5218,22 +5218,22 @@
       </c>
       <c r="Z40" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA40" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
-          <t>80.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC40" s="2" t="inlineStr">
         <is>
-          <t>14/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
@@ -5337,22 +5337,22 @@
       </c>
       <c r="Z41" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA41" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>77.9</t>
         </is>
       </c>
       <c r="AC41" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>4/15</t>
         </is>
       </c>
     </row>
@@ -5417,7 +5417,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -5461,17 +5461,17 @@
       </c>
       <c r="AA42" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>77.2</t>
         </is>
       </c>
       <c r="AC42" s="2" t="inlineStr">
         <is>
-          <t>2/15</t>
+          <t>3/15</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
@@ -5580,17 +5580,17 @@
       </c>
       <c r="AA43" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
-          <t>78.6</t>
+          <t>81.8</t>
         </is>
       </c>
       <c r="AC43" s="2" t="inlineStr">
         <is>
-          <t>6/15</t>
+          <t>13/15</t>
         </is>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5694,22 +5694,22 @@
       </c>
       <c r="Z44" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA44" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="AC44" s="2" t="inlineStr">
         <is>
-          <t>1/15</t>
+          <t>2/15</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -5813,22 +5813,22 @@
       </c>
       <c r="Z45" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA45" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC45" s="2" t="inlineStr">
         <is>
-          <t>5/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -5932,22 +5932,22 @@
       </c>
       <c r="Z46" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA46" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC46" s="2" t="inlineStr">
         <is>
-          <t>7/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -6056,12 +6056,12 @@
       </c>
       <c r="AA47" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
-          <t>83.8</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="AC47" s="2" t="inlineStr">
@@ -6131,7 +6131,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -6170,22 +6170,22 @@
       </c>
       <c r="Z48" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA48" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
-          <t>80.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC48" s="2" t="inlineStr">
         <is>
-          <t>14/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -6250,7 +6250,7 @@
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="P49" s="2" t="inlineStr">
@@ -6299,12 +6299,12 @@
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
-          <t>79.9</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="AC49" s="2" t="inlineStr">
         <is>
-          <t>9/15</t>
+          <t>8/15</t>
         </is>
       </c>
     </row>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -6413,17 +6413,17 @@
       </c>
       <c r="AA50" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>77.2</t>
         </is>
       </c>
       <c r="AC50" s="2" t="inlineStr">
         <is>
-          <t>2/15</t>
+          <t>3/15</t>
         </is>
       </c>
     </row>
@@ -6488,7 +6488,7 @@
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="P51" s="2" t="inlineStr">
@@ -6527,22 +6527,22 @@
       </c>
       <c r="Z51" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA51" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>82.7</t>
         </is>
       </c>
       <c r="AC51" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>14/15</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -6646,22 +6646,22 @@
       </c>
       <c r="Z52" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA52" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="AC52" s="2" t="inlineStr">
         <is>
-          <t>1/15</t>
+          <t>2/15</t>
         </is>
       </c>
     </row>
@@ -6776,7 +6776,7 @@
       </c>
       <c r="AC53" s="2" t="inlineStr">
         <is>
-          <t>8/15</t>
+          <t>9/15</t>
         </is>
       </c>
     </row>
@@ -6841,7 +6841,7 @@
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
@@ -6880,22 +6880,22 @@
       </c>
       <c r="Z54" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AA54" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>78.2</t>
         </is>
       </c>
       <c r="AC54" s="2" t="inlineStr">
         <is>
-          <t>3/15</t>
+          <t>5/15</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
@@ -7004,12 +7004,12 @@
       </c>
       <c r="AA55" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
-          <t>83.8</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="AC55" s="2" t="inlineStr">
@@ -7079,7 +7079,7 @@
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="P56" s="2" t="inlineStr">
@@ -7118,22 +7118,22 @@
       </c>
       <c r="Z56" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA56" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="AC56" s="2" t="inlineStr">
         <is>
-          <t>4/15</t>
+          <t>1/15</t>
         </is>
       </c>
     </row>
@@ -7198,7 +7198,7 @@
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="P57" s="2" t="inlineStr">
@@ -7247,12 +7247,12 @@
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
-          <t>79.9</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="AC57" s="2" t="inlineStr">
         <is>
-          <t>9/15</t>
+          <t>8/15</t>
         </is>
       </c>
     </row>
@@ -7317,7 +7317,7 @@
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P58" s="2" t="inlineStr">
@@ -7356,22 +7356,22 @@
       </c>
       <c r="Z58" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA58" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
-          <t>80.4</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC58" s="2" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -7490,7 +7490,7 @@
       </c>
       <c r="AC59" s="2" t="inlineStr">
         <is>
-          <t>13/15</t>
+          <t>12/15</t>
         </is>
       </c>
     </row>
@@ -7555,7 +7555,7 @@
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="P60" s="2" t="inlineStr">
@@ -7594,22 +7594,22 @@
       </c>
       <c r="Z60" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA60" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>82.7</t>
         </is>
       </c>
       <c r="AC60" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>14/15</t>
         </is>
       </c>
     </row>
@@ -7674,7 +7674,7 @@
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P61" s="2" t="inlineStr">
@@ -7713,22 +7713,22 @@
       </c>
       <c r="Z61" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA61" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>77.9</t>
         </is>
       </c>
       <c r="AC61" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>4/15</t>
         </is>
       </c>
     </row>
@@ -7793,7 +7793,7 @@
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr">
@@ -7832,22 +7832,22 @@
       </c>
       <c r="Z62" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AA62" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>78.2</t>
         </is>
       </c>
       <c r="AC62" s="2" t="inlineStr">
         <is>
-          <t>3/15</t>
+          <t>5/15</t>
         </is>
       </c>
     </row>
@@ -7912,7 +7912,7 @@
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P63" s="2" t="inlineStr">
@@ -7951,22 +7951,22 @@
       </c>
       <c r="Z63" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA63" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC63" s="2" t="inlineStr">
         <is>
-          <t>5/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -8031,7 +8031,7 @@
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="P64" s="2" t="inlineStr">
@@ -8070,22 +8070,22 @@
       </c>
       <c r="Z64" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA64" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="AC64" s="2" t="inlineStr">
         <is>
-          <t>4/15</t>
+          <t>1/15</t>
         </is>
       </c>
     </row>
@@ -8150,7 +8150,7 @@
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="P65" s="2" t="inlineStr">
@@ -8194,17 +8194,17 @@
       </c>
       <c r="AA65" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
-          <t>78.6</t>
+          <t>81.8</t>
         </is>
       </c>
       <c r="AC65" s="2" t="inlineStr">
         <is>
-          <t>6/15</t>
+          <t>13/15</t>
         </is>
       </c>
     </row>
@@ -8269,7 +8269,7 @@
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P66" s="2" t="inlineStr">
@@ -8308,22 +8308,22 @@
       </c>
       <c r="Z66" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA66" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC66" s="2" t="inlineStr">
         <is>
-          <t>7/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -8388,7 +8388,7 @@
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P67" s="2" t="inlineStr">
@@ -8427,22 +8427,22 @@
       </c>
       <c r="Z67" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA67" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
-          <t>80.4</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC67" s="2" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -8507,7 +8507,7 @@
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P68" s="2" t="inlineStr">
@@ -8546,22 +8546,22 @@
       </c>
       <c r="Z68" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA68" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
-          <t>80.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC68" s="2" t="inlineStr">
         <is>
-          <t>14/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -8680,7 +8680,7 @@
       </c>
       <c r="AC69" s="2" t="inlineStr">
         <is>
-          <t>13/15</t>
+          <t>12/15</t>
         </is>
       </c>
     </row>
@@ -8745,7 +8745,7 @@
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="P70" s="2" t="inlineStr">
@@ -8789,12 +8789,12 @@
       </c>
       <c r="AA70" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
-          <t>83.8</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="AC70" s="2" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="P71" s="2" t="inlineStr">
@@ -8913,12 +8913,12 @@
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
-          <t>79.9</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="AC71" s="2" t="inlineStr">
         <is>
-          <t>9/15</t>
+          <t>8/15</t>
         </is>
       </c>
     </row>
@@ -8983,7 +8983,7 @@
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P72" s="2" t="inlineStr">
@@ -9022,22 +9022,22 @@
       </c>
       <c r="Z72" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA72" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>77.9</t>
         </is>
       </c>
       <c r="AC72" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>4/15</t>
         </is>
       </c>
     </row>
@@ -9070,27 +9070,31 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>84分钟</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr"/>
       <c r="K73" s="2" t="inlineStr"/>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M73" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
           <t>07:21</t>
@@ -9098,7 +9102,7 @@
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="P73" s="2" t="inlineStr">
@@ -9122,17 +9126,17 @@
       </c>
       <c r="W73" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X73" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y73" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z73" s="2" t="inlineStr">
@@ -9142,17 +9146,17 @@
       </c>
       <c r="AA73" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>77.2</t>
         </is>
       </c>
       <c r="AC73" s="2" t="inlineStr">
         <is>
-          <t>2/15</t>
+          <t>3/15</t>
         </is>
       </c>
     </row>
@@ -9185,27 +9189,31 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>90分钟</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M74" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
           <t>06:11</t>
@@ -9213,7 +9221,7 @@
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P74" s="2" t="inlineStr">
@@ -9237,37 +9245,37 @@
       </c>
       <c r="W74" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X74" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y74" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z74" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA74" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC74" s="2" t="inlineStr">
         <is>
-          <t>5/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -9300,24 +9308,24 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>82分钟</t>
+          <t>94分钟</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr"/>
       <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数82分钟估算，约±5分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M75" s="2" t="inlineStr">
@@ -9332,7 +9340,7 @@
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="P75" s="2" t="inlineStr">
@@ -9356,12 +9364,12 @@
       </c>
       <c r="W75" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X75" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y75" s="2" t="inlineStr">
@@ -9371,22 +9379,22 @@
       </c>
       <c r="Z75" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA75" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>82.7</t>
         </is>
       </c>
       <c r="AC75" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>14/15</t>
         </is>
       </c>
     </row>
@@ -9419,27 +9427,31 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>18:46</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>91分钟</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M76" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
           <t>07:51</t>
@@ -9447,7 +9459,7 @@
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="P76" s="2" t="inlineStr">
@@ -9471,37 +9483,37 @@
       </c>
       <c r="W76" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X76" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y76" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z76" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA76" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="AC76" s="2" t="inlineStr">
         <is>
-          <t>1/15</t>
+          <t>2/15</t>
         </is>
       </c>
     </row>
@@ -9534,27 +9546,31 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>98分钟</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M77" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -9562,7 +9578,7 @@
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="P77" s="2" t="inlineStr">
@@ -9586,17 +9602,17 @@
       </c>
       <c r="W77" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X77" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y77" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z77" s="2" t="inlineStr">
@@ -9606,17 +9622,17 @@
       </c>
       <c r="AA77" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
-          <t>78.6</t>
+          <t>81.8</t>
         </is>
       </c>
       <c r="AC77" s="2" t="inlineStr">
         <is>
-          <t>6/15</t>
+          <t>13/15</t>
         </is>
       </c>
     </row>
@@ -9649,27 +9665,31 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>98分钟</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M78" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
           <t>06:41</t>
@@ -9677,7 +9697,7 @@
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P78" s="2" t="inlineStr">
@@ -9701,37 +9721,37 @@
       </c>
       <c r="W78" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X78" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y78" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z78" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA78" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC78" s="2" t="inlineStr">
         <is>
-          <t>7/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -9764,27 +9784,31 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>83分钟</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
       <c r="K79" s="2" t="inlineStr"/>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M79" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
           <t>13:31</t>
@@ -9792,7 +9816,7 @@
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="P79" s="2" t="inlineStr">
@@ -9816,37 +9840,37 @@
       </c>
       <c r="W79" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X79" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y79" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z79" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AA79" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>78.2</t>
         </is>
       </c>
       <c r="AC79" s="2" t="inlineStr">
         <is>
-          <t>3/15</t>
+          <t>5/15</t>
         </is>
       </c>
     </row>
@@ -9879,27 +9903,31 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>91分钟</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M80" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
           <t>07:11</t>
@@ -9907,7 +9935,7 @@
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P80" s="2" t="inlineStr">
@@ -9931,37 +9959,37 @@
       </c>
       <c r="W80" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X80" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y80" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z80" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA80" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
-          <t>80.8</t>
+          <t>79.9</t>
         </is>
       </c>
       <c r="AC80" s="2" t="inlineStr">
         <is>
-          <t>14/15</t>
+          <t>10/15</t>
         </is>
       </c>
     </row>
@@ -9994,27 +10022,31 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>81分钟</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr"/>
       <c r="K81" s="2" t="inlineStr"/>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M81" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -10022,7 +10054,7 @@
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
@@ -10046,37 +10078,37 @@
       </c>
       <c r="W81" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X81" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y81" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z81" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA81" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="AC81" s="2" t="inlineStr">
         <is>
-          <t>4/15</t>
+          <t>1/15</t>
         </is>
       </c>
     </row>
@@ -10109,27 +10141,31 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>85分钟</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr"/>
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M82" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -10137,7 +10173,7 @@
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="P82" s="2" t="inlineStr">
@@ -10161,17 +10197,17 @@
       </c>
       <c r="W82" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X82" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y82" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z82" s="2" t="inlineStr">
@@ -10181,12 +10217,12 @@
       </c>
       <c r="AA82" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
-          <t>83.8</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="AC82" s="2" t="inlineStr">
@@ -10224,29 +10260,29 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>19:42</t>
+          <t>19:39</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>88分钟</t>
+          <t>84分钟</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr"/>
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数88分钟估算，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M83" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N83" s="2" t="inlineStr">
@@ -10256,7 +10292,7 @@
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="P83" s="2" t="inlineStr">
@@ -10280,12 +10316,12 @@
       </c>
       <c r="W83" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X83" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y83" s="2" t="inlineStr">
@@ -10305,12 +10341,12 @@
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
-          <t>79.9</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="AC83" s="2" t="inlineStr">
         <is>
-          <t>9/15</t>
+          <t>8/15</t>
         </is>
       </c>
     </row>
@@ -10343,29 +10379,29 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:37</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>88分钟</t>
+          <t>82分钟</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
       <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数88分钟估算，约±7分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
         </is>
       </c>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N84" s="2" t="inlineStr">
@@ -10375,7 +10411,7 @@
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P84" s="2" t="inlineStr">
@@ -10399,12 +10435,12 @@
       </c>
       <c r="W84" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X84" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y84" s="2" t="inlineStr">
@@ -10414,22 +10450,22 @@
       </c>
       <c r="Z84" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA84" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
-          <t>80.4</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="AC84" s="2" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>6/15</t>
         </is>
       </c>
     </row>
@@ -10462,27 +10498,31 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>19:51</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>80分钟</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
       <c r="K85" s="2" t="inlineStr"/>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M85" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N85" s="2" t="inlineStr">
         <is>
           <t>07:21</t>
@@ -10490,7 +10530,7 @@
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="P85" s="2" t="inlineStr">
@@ -10514,17 +10554,17 @@
       </c>
       <c r="W85" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X85" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y85" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z85" s="2" t="inlineStr">
@@ -10534,17 +10574,17 @@
       </c>
       <c r="AA85" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>77.2</t>
         </is>
       </c>
       <c r="AC85" s="2" t="inlineStr">
         <is>
-          <t>2/15</t>
+          <t>3/15</t>
         </is>
       </c>
     </row>
@@ -10577,27 +10617,31 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>19:52</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M86" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -10605,7 +10649,7 @@
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="P86" s="2" t="inlineStr">
@@ -10629,37 +10673,37 @@
       </c>
       <c r="W86" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X86" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y86" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z86" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AA86" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
-          <t>80.3</t>
+          <t>77.9</t>
         </is>
       </c>
       <c r="AC86" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>4/15</t>
         </is>
       </c>
     </row>
@@ -10667,24 +10711,24 @@
       <c r="A87" s="2" t="inlineStr"/>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>沪A67983D</t>
+          <t>沪A68397D</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
           <t>川沙客运站</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>19:05</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>金杨路金口路</t>
-        </is>
-      </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -10692,35 +10736,39 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>85分钟</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr"/>
       <c r="K87" s="2" t="inlineStr"/>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M87" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>06:02</t>
         </is>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="P87" s="2" t="inlineStr">
@@ -10734,47 +10782,1348 @@
       <c r="T87" s="2" t="inlineStr"/>
       <c r="U87" s="2" t="inlineStr">
         <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="V87" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W87" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X87" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y87" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z87" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AA87" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AB87" s="2" t="inlineStr">
+        <is>
+          <t>82.7</t>
+        </is>
+      </c>
+      <c r="AC87" s="2" t="inlineStr">
+        <is>
+          <t>14/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr"/>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>沪A08953A</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>76分钟</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>20:12</t>
+        </is>
+      </c>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q88" s="2" t="inlineStr"/>
+      <c r="R88" s="2" t="inlineStr"/>
+      <c r="S88" s="2" t="inlineStr"/>
+      <c r="T88" s="2" t="inlineStr"/>
+      <c r="U88" s="2" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="V88" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W88" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X88" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y88" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z88" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AA88" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AB88" s="2" t="inlineStr">
+        <is>
+          <t>77.0</t>
+        </is>
+      </c>
+      <c r="AC88" s="2" t="inlineStr">
+        <is>
+          <t>2/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr"/>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
           <t>19:05</t>
         </is>
       </c>
-      <c r="V87" s="2" t="inlineStr">
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>81分钟</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr"/>
+      <c r="K89" s="2" t="inlineStr"/>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="P89" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q89" s="2" t="inlineStr"/>
+      <c r="R89" s="2" t="inlineStr"/>
+      <c r="S89" s="2" t="inlineStr"/>
+      <c r="T89" s="2" t="inlineStr"/>
+      <c r="U89" s="2" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="V89" s="2" t="inlineStr">
         <is>
           <t>计划发车</t>
         </is>
       </c>
-      <c r="W87" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="X87" s="2" t="inlineStr">
-        <is>
-          <t>证据不足</t>
-        </is>
-      </c>
-      <c r="Y87" s="2" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="Z87" s="2" t="inlineStr">
+      <c r="W89" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X89" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y89" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z89" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AA89" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AB89" s="2" t="inlineStr">
+        <is>
+          <t>78.8</t>
+        </is>
+      </c>
+      <c r="AC89" s="2" t="inlineStr">
+        <is>
+          <t>6/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr"/>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>80分钟</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr"/>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>20:31</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q90" s="2" t="inlineStr"/>
+      <c r="R90" s="2" t="inlineStr"/>
+      <c r="S90" s="2" t="inlineStr"/>
+      <c r="T90" s="2" t="inlineStr"/>
+      <c r="U90" s="2" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="V90" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W90" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X90" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y90" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z90" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AA90" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AB90" s="2" t="inlineStr">
+        <is>
+          <t>78.2</t>
+        </is>
+      </c>
+      <c r="AC90" s="2" t="inlineStr">
+        <is>
+          <t>5/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr"/>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>20:43</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>73分钟</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr"/>
+      <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="P91" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q91" s="2" t="inlineStr"/>
+      <c r="R91" s="2" t="inlineStr"/>
+      <c r="S91" s="2" t="inlineStr"/>
+      <c r="T91" s="2" t="inlineStr"/>
+      <c r="U91" s="2" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="V91" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W91" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X91" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y91" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z91" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AA91" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AB91" s="2" t="inlineStr">
+        <is>
+          <t>79.9</t>
+        </is>
+      </c>
+      <c r="AC91" s="2" t="inlineStr">
+        <is>
+          <t>10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr"/>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>75分钟</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>20:31</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q92" s="2" t="inlineStr"/>
+      <c r="R92" s="2" t="inlineStr"/>
+      <c r="S92" s="2" t="inlineStr"/>
+      <c r="T92" s="2" t="inlineStr"/>
+      <c r="U92" s="2" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="V92" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W92" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X92" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y92" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z92" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="AA87" s="2" t="inlineStr">
+      <c r="AA92" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AB92" s="2" t="inlineStr">
+        <is>
+          <t>76.7</t>
+        </is>
+      </c>
+      <c r="AC92" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr"/>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>73分钟</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr"/>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS末次终点ETA推算：20:51采样，终点ETA 11分钟</t>
+        </is>
+      </c>
+      <c r="M93" s="2" t="inlineStr"/>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="P93" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q93" s="2" t="inlineStr"/>
+      <c r="R93" s="2" t="inlineStr"/>
+      <c r="S93" s="2" t="inlineStr"/>
+      <c r="T93" s="2" t="inlineStr"/>
+      <c r="U93" s="2" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="V93" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W93" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X93" s="2" t="inlineStr">
+        <is>
+          <t>末次终点ETA兜底</t>
+        </is>
+      </c>
+      <c r="Y93" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z93" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AA93" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AB93" s="2" t="inlineStr">
+        <is>
+          <t>78.8</t>
+        </is>
+      </c>
+      <c r="AC93" s="2" t="inlineStr">
+        <is>
+          <t>6/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr"/>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>72分钟</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="P94" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q94" s="2" t="inlineStr"/>
+      <c r="R94" s="2" t="inlineStr"/>
+      <c r="S94" s="2" t="inlineStr"/>
+      <c r="T94" s="2" t="inlineStr"/>
+      <c r="U94" s="2" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="V94" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W94" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X94" s="2" t="inlineStr">
+        <is>
+          <t>终点ETA确认/一致估算</t>
+        </is>
+      </c>
+      <c r="Y94" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z94" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AA94" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AB94" s="2" t="inlineStr">
+        <is>
+          <t>79.9</t>
+        </is>
+      </c>
+      <c r="AC94" s="2" t="inlineStr">
+        <is>
+          <t>10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr"/>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>20:10</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>21:18</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>69分钟</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr"/>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS末次终点ETA推算：20:51采样，终点ETA 27分钟</t>
+        </is>
+      </c>
+      <c r="M95" s="2" t="inlineStr"/>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="P95" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q95" s="2" t="inlineStr"/>
+      <c r="R95" s="2" t="inlineStr"/>
+      <c r="S95" s="2" t="inlineStr"/>
+      <c r="T95" s="2" t="inlineStr"/>
+      <c r="U95" s="2" t="inlineStr">
+        <is>
+          <t>20:10</t>
+        </is>
+      </c>
+      <c r="V95" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W95" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X95" s="2" t="inlineStr">
+        <is>
+          <t>末次终点ETA兜底</t>
+        </is>
+      </c>
+      <c r="Y95" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z95" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AA95" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AB95" s="2" t="inlineStr">
+        <is>
+          <t>77.9</t>
+        </is>
+      </c>
+      <c r="AC95" s="2" t="inlineStr">
+        <is>
+          <t>4/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr"/>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>21:42</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>73分钟</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>20:51采样：该车到重点站东陆路新金桥路 ETA 9分钟；叠加该车自身同类时段从该站到终点历史中位数42分钟，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="AB87" s="2" t="inlineStr">
-        <is>
-          <t>77.2</t>
-        </is>
-      </c>
-      <c r="AC87" s="2" t="inlineStr">
-        <is>
-          <t>5/15</t>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="P96" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q96" s="2" t="inlineStr"/>
+      <c r="R96" s="2" t="inlineStr"/>
+      <c r="S96" s="2" t="inlineStr"/>
+      <c r="T96" s="2" t="inlineStr"/>
+      <c r="U96" s="2" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="V96" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W96" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X96" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y96" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z96" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AA96" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AB96" s="2" t="inlineStr">
+        <is>
+          <t>78.8</t>
+        </is>
+      </c>
+      <c r="AC96" s="2" t="inlineStr">
+        <is>
+          <t>6/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr"/>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>74分钟</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr"/>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数74分钟估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="O97" s="2" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="P97" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q97" s="2" t="inlineStr"/>
+      <c r="R97" s="2" t="inlineStr"/>
+      <c r="S97" s="2" t="inlineStr"/>
+      <c r="T97" s="2" t="inlineStr"/>
+      <c r="U97" s="2" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="V97" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W97" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X97" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y97" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z97" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AA97" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AB97" s="2" t="inlineStr">
+        <is>
+          <t>79.9</t>
+        </is>
+      </c>
+      <c r="AC97" s="2" t="inlineStr">
+        <is>
+          <t>10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr"/>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>22:27</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>72分钟</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数72分钟估算，约±6分钟</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q98" s="2" t="inlineStr"/>
+      <c r="R98" s="2" t="inlineStr"/>
+      <c r="S98" s="2" t="inlineStr"/>
+      <c r="T98" s="2" t="inlineStr"/>
+      <c r="U98" s="2" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="V98" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W98" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X98" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y98" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z98" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AA98" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AB98" s="2" t="inlineStr">
+        <is>
+          <t>79.9</t>
+        </is>
+      </c>
+      <c r="AC98" s="2" t="inlineStr">
+        <is>
+          <t>10/15</t>
         </is>
       </c>
     </row>

</xml_diff>